<commit_message>
Fix stock variance template formulas and default currency
</commit_message>
<xml_diff>
--- a/downloads/inventory/dixani-stock-variance-report.xlsx
+++ b/downloads/inventory/dixani-stock-variance-report.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Variance Report" sheetId="1" r:id="Rdfcfc845abc64d11"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="How to Use" sheetId="2" r:id="R135fd6acb31b418e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Example" sheetId="3" r:id="R5eb3fe7edb434922"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Variance Report" sheetId="1" r:id="R0eacd5cfc2a64b92"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="How to Use" sheetId="2" r:id="Rb00bdc3fbaa4468f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Example" sheetId="3" r:id="R751dc50622734a4b"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -21,7 +21,7 @@
     <x:numFmt numFmtId="202" formatCode="#,##0.00"/>
     <x:numFmt numFmtId="203" formatCode="yyyy-mm-dd"/>
   </x:numFmts>
-  <x:fonts count="8">
+  <x:fonts count="9">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -68,6 +68,11 @@
       <x:color rgb="FFFFFFFF"/>
       <x:name val="Carlito"/>
     </x:font>
+    <x:font>
+      <x:sz val="10"/>
+      <x:color rgb="FF475569"/>
+      <x:name val="Carlito"/>
+    </x:font>
   </x:fonts>
   <x:fills count="6">
     <x:fill>
@@ -104,7 +109,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="69">
+  <x:cellXfs count="72">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -258,18 +263,25 @@
       <x:alignment horizontal="center"/>
     </x:xf>
     <x:xf numFmtId="202" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
   </x:cellStyles>
-  <x:dxfs count="3">
+  <x:dxfs count="4">
     <x:dxf>
       <x:font>
         <x:b/>
         <x:color rgb="FF15803D"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFDCFCE7"/>
         </x:patternFill>
       </x:fill>
@@ -280,7 +292,7 @@
         <x:color rgb="FFB91C1C"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFEE2E2"/>
         </x:patternFill>
       </x:fill>
@@ -291,8 +303,18 @@
         <x:color rgb="FF92400E"/>
       </x:font>
       <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEF3C7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:color rgb="FF92400E"/>
+      </x:font>
+      <x:fill>
         <x:patternFill patternType="solid">
-          <x:bgColor rgb="FFFEF3C7"/>
+          <x:bgColor rgb="FFFFF3CD"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
@@ -495,7 +517,7 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="5" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="11" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="18" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="27" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="15" hidden="0" customWidth="1"/>
@@ -572,7 +594,7 @@
         <x:v>Currency</x:v>
       </x:c>
       <x:c r="B5" t="str">
-        <x:v>QAR</x:v>
+        <x:v>USD</x:v>
       </x:c>
       <x:c r="C5" t="str"/>
       <x:c r="D5" s="16" t="str">
@@ -611,7 +633,7 @@
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="23" t="str">
-        <x:v>Total Items</x:v>
+        <x:v>Started Rows</x:v>
       </x:c>
       <x:c r="B8" s="23" t="str"/>
       <x:c r="C8" s="23" t="str">
@@ -638,10 +660,10 @@
         <x:v>Net Variance Value</x:v>
       </x:c>
     </x:row>
-    <x:row r="9">
+    <x:row r="9" ht="28" customHeight="1">
       <x:c r="A9" s="29" t="n">
-        <x:f>COUNTIF(M13:M52,"&lt;&gt;")</x:f>
-        <x:v>40</x:v>
+        <x:f>COUNT(I13:I52)+COUNTIF(M13:M52,"INCOMPLETE")</x:f>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="B9" s="29"/>
       <x:c r="C9" s="29" t="n">
@@ -660,19 +682,37 @@
       </x:c>
       <x:c r="H9" s="29"/>
       <x:c r="I9" s="60" t="n">
-        <x:f>-SUMIF(L13:L52,"&lt;0",L13:L52)</x:f>
+        <x:f>IF(A9&lt;&gt;COUNT(L13:L52),"Incomplete",-SUMIF(L13:L52,"&lt;0",L13:L52))</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="J9" s="60"/>
       <x:c r="K9" s="60" t="n">
-        <x:f>SUMIF(L13:L52,"&gt;0",L13:L52)</x:f>
+        <x:f>IF(A9&lt;&gt;COUNT(L13:L52),"Incomplete",SUMIF(L13:L52,"&gt;0",L13:L52))</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="L9" s="60"/>
       <x:c r="M9" s="60" t="n">
-        <x:f>SUM(L13:L52)</x:f>
+        <x:f>IF(A9&lt;&gt;COUNT(L13:L52),"Incomplete",SUM(L13:L52))</x:f>
         <x:v>0</x:v>
       </x:c>
+    </x:row>
+    <x:row r="10" ht="24" customHeight="1">
+      <x:c r="A10" s="69" t="str">
+        <x:f>"Rows needing quantities: "&amp;COUNTIF(M13:M52,"INCOMPLETE")&amp;". Value totals require valid quantities and costs for every started row."</x:f>
+        <x:v>Rows needing quantities: 0. Value totals require valid quantities and costs for every started row.</x:v>
+      </x:c>
+      <x:c r="B10" s="69"/>
+      <x:c r="C10" s="69"/>
+      <x:c r="D10" s="69"/>
+      <x:c r="E10" s="69"/>
+      <x:c r="F10" s="69"/>
+      <x:c r="G10" s="69"/>
+      <x:c r="H10" s="69"/>
+      <x:c r="I10" s="69"/>
+      <x:c r="J10" s="69"/>
+      <x:c r="K10" s="69"/>
+      <x:c r="L10" s="69"/>
+      <x:c r="M10" s="69"/>
     </x:row>
     <x:row r="12" ht="32" customHeight="1">
       <x:c r="A12" s="35" t="str">
@@ -719,50 +759,50 @@
       <x:c r="A13" s="40" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="B13" s="40" t="str"/>
-      <x:c r="C13" s="40" t="str"/>
-      <x:c r="D13" s="40" t="str"/>
-      <x:c r="E13" s="40" t="str"/>
-      <x:c r="F13" s="40" t="str"/>
-      <x:c r="G13" s="48" t="str"/>
-      <x:c r="H13" s="48" t="str"/>
+      <x:c r="B13" s="40"/>
+      <x:c r="C13" s="40"/>
+      <x:c r="D13" s="40"/>
+      <x:c r="E13" s="40"/>
+      <x:c r="F13" s="40"/>
+      <x:c r="G13" s="48"/>
+      <x:c r="H13" s="48"/>
       <x:c r="I13" s="48" t="str">
-        <x:f>IF(OR(G13="",H13=""),"",H13-G13)</x:f>
+        <x:f>IF(AND(ISNUMBER(G13),ISNUMBER(H13),G13&gt;=0,H13&gt;=0),H13-G13,"")</x:f>
       </x:c>
       <x:c r="J13" s="52" t="str">
-        <x:f>IF(OR(G13="",H13=""),"",IF(G13=0,IF(H13=0,0,1),I13/G13))</x:f>
-      </x:c>
-      <x:c r="K13" s="56" t="str"/>
+        <x:f>IF(ISNUMBER(I13),IF(G13=0,"N/A",I13/G13),"")</x:f>
+      </x:c>
+      <x:c r="K13" s="56"/>
       <x:c r="L13" s="56" t="str">
-        <x:f>IF(OR(I13="",K13=""),"",I13*K13)</x:f>
+        <x:f>IF(AND(ISNUMBER(I13),ISNUMBER(K13),K13&gt;=0),I13*K13,"")</x:f>
       </x:c>
       <x:c r="M13" s="40" t="str">
-        <x:f>IF(I13="","",IF(I13=0,"MATCHED",IF(I13&lt;0,"SHORTAGE","EXCESS")))</x:f>
+        <x:f>IF(COUNTA(B13:H13,K13)=0,"",IF(ISNUMBER(I13),IF(I13=0,"MATCHED",IF(I13&lt;0,"SHORTAGE","EXCESS")),"INCOMPLETE"))</x:f>
       </x:c>
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="42" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="B14" s="42" t="str"/>
-      <x:c r="C14" s="42" t="str"/>
-      <x:c r="D14" s="42" t="str"/>
-      <x:c r="E14" s="42" t="str"/>
-      <x:c r="F14" s="42" t="str"/>
-      <x:c r="G14" s="49" t="str"/>
-      <x:c r="H14" s="49" t="str"/>
+      <x:c r="B14" s="42"/>
+      <x:c r="C14" s="42"/>
+      <x:c r="D14" s="42"/>
+      <x:c r="E14" s="42"/>
+      <x:c r="F14" s="42"/>
+      <x:c r="G14" s="49"/>
+      <x:c r="H14" s="49"/>
       <x:c r="I14" s="49" t="str">
-        <x:f>IF(OR(G14="",H14=""),"",H14-G14)</x:f>
+        <x:f>IF(AND(ISNUMBER(G14),ISNUMBER(H14),G14&gt;=0,H14&gt;=0),H14-G14,"")</x:f>
       </x:c>
       <x:c r="J14" s="53" t="str">
-        <x:f>IF(OR(G14="",H14=""),"",IF(G14=0,IF(H14=0,0,1),I14/G14))</x:f>
-      </x:c>
-      <x:c r="K14" s="57" t="str"/>
+        <x:f>IF(ISNUMBER(I14),IF(G14=0,"N/A",I14/G14),"")</x:f>
+      </x:c>
+      <x:c r="K14" s="57"/>
       <x:c r="L14" s="57" t="str">
-        <x:f>IF(OR(I14="",K14=""),"",I14*K14)</x:f>
+        <x:f>IF(AND(ISNUMBER(I14),ISNUMBER(K14),K14&gt;=0),I14*K14,"")</x:f>
       </x:c>
       <x:c r="M14" s="42" t="str">
-        <x:f>IF(I14="","",IF(I14=0,"MATCHED",IF(I14&lt;0,"SHORTAGE","EXCESS")))</x:f>
+        <x:f>IF(COUNTA(B14:H14,K14)=0,"",IF(ISNUMBER(I14),IF(I14=0,"MATCHED",IF(I14&lt;0,"SHORTAGE","EXCESS")),"INCOMPLETE"))</x:f>
       </x:c>
     </x:row>
     <x:row r="15">
@@ -777,17 +817,17 @@
       <x:c r="G15" s="48" t="str"/>
       <x:c r="H15" s="48" t="str"/>
       <x:c r="I15" s="48" t="str">
-        <x:f>IF(OR(G15="",H15=""),"",H15-G15)</x:f>
+        <x:f>IF(AND(ISNUMBER(G15),ISNUMBER(H15),G15&gt;=0,H15&gt;=0),H15-G15,"")</x:f>
       </x:c>
       <x:c r="J15" s="52" t="str">
-        <x:f>IF(OR(G15="",H15=""),"",IF(G15=0,IF(H15=0,0,1),I15/G15))</x:f>
+        <x:f>IF(ISNUMBER(I15),IF(G15=0,"N/A",I15/G15),"")</x:f>
       </x:c>
       <x:c r="K15" s="56" t="str"/>
       <x:c r="L15" s="56" t="str">
-        <x:f>IF(OR(I15="",K15=""),"",I15*K15)</x:f>
+        <x:f>IF(AND(ISNUMBER(I15),ISNUMBER(K15),K15&gt;=0),I15*K15,"")</x:f>
       </x:c>
       <x:c r="M15" s="40" t="str">
-        <x:f>IF(I15="","",IF(I15=0,"MATCHED",IF(I15&lt;0,"SHORTAGE","EXCESS")))</x:f>
+        <x:f>IF(COUNTA(B15:H15,K15)=0,"",IF(ISNUMBER(I15),IF(I15=0,"MATCHED",IF(I15&lt;0,"SHORTAGE","EXCESS")),"INCOMPLETE"))</x:f>
       </x:c>
     </x:row>
     <x:row r="16">
@@ -802,17 +842,17 @@
       <x:c r="G16" s="49" t="str"/>
       <x:c r="H16" s="49" t="str"/>
       <x:c r="I16" s="49" t="str">
-        <x:f>IF(OR(G16="",H16=""),"",H16-G16)</x:f>
+        <x:f>IF(AND(ISNUMBER(G16),ISNUMBER(H16),G16&gt;=0,H16&gt;=0),H16-G16,"")</x:f>
       </x:c>
       <x:c r="J16" s="53" t="str">
-        <x:f>IF(OR(G16="",H16=""),"",IF(G16=0,IF(H16=0,0,1),I16/G16))</x:f>
+        <x:f>IF(ISNUMBER(I16),IF(G16=0,"N/A",I16/G16),"")</x:f>
       </x:c>
       <x:c r="K16" s="57" t="str"/>
       <x:c r="L16" s="57" t="str">
-        <x:f>IF(OR(I16="",K16=""),"",I16*K16)</x:f>
+        <x:f>IF(AND(ISNUMBER(I16),ISNUMBER(K16),K16&gt;=0),I16*K16,"")</x:f>
       </x:c>
       <x:c r="M16" s="42" t="str">
-        <x:f>IF(I16="","",IF(I16=0,"MATCHED",IF(I16&lt;0,"SHORTAGE","EXCESS")))</x:f>
+        <x:f>IF(COUNTA(B16:H16,K16)=0,"",IF(ISNUMBER(I16),IF(I16=0,"MATCHED",IF(I16&lt;0,"SHORTAGE","EXCESS")),"INCOMPLETE"))</x:f>
       </x:c>
     </x:row>
     <x:row r="17">
@@ -827,17 +867,17 @@
       <x:c r="G17" s="48" t="str"/>
       <x:c r="H17" s="48" t="str"/>
       <x:c r="I17" s="48" t="str">
-        <x:f>IF(OR(G17="",H17=""),"",H17-G17)</x:f>
+        <x:f>IF(AND(ISNUMBER(G17),ISNUMBER(H17),G17&gt;=0,H17&gt;=0),H17-G17,"")</x:f>
       </x:c>
       <x:c r="J17" s="52" t="str">
-        <x:f>IF(OR(G17="",H17=""),"",IF(G17=0,IF(H17=0,0,1),I17/G17))</x:f>
+        <x:f>IF(ISNUMBER(I17),IF(G17=0,"N/A",I17/G17),"")</x:f>
       </x:c>
       <x:c r="K17" s="56" t="str"/>
       <x:c r="L17" s="56" t="str">
-        <x:f>IF(OR(I17="",K17=""),"",I17*K17)</x:f>
+        <x:f>IF(AND(ISNUMBER(I17),ISNUMBER(K17),K17&gt;=0),I17*K17,"")</x:f>
       </x:c>
       <x:c r="M17" s="40" t="str">
-        <x:f>IF(I17="","",IF(I17=0,"MATCHED",IF(I17&lt;0,"SHORTAGE","EXCESS")))</x:f>
+        <x:f>IF(COUNTA(B17:H17,K17)=0,"",IF(ISNUMBER(I17),IF(I17=0,"MATCHED",IF(I17&lt;0,"SHORTAGE","EXCESS")),"INCOMPLETE"))</x:f>
       </x:c>
     </x:row>
     <x:row r="18">
@@ -852,17 +892,17 @@
       <x:c r="G18" s="49" t="str"/>
       <x:c r="H18" s="49" t="str"/>
       <x:c r="I18" s="49" t="str">
-        <x:f>IF(OR(G18="",H18=""),"",H18-G18)</x:f>
+        <x:f>IF(AND(ISNUMBER(G18),ISNUMBER(H18),G18&gt;=0,H18&gt;=0),H18-G18,"")</x:f>
       </x:c>
       <x:c r="J18" s="53" t="str">
-        <x:f>IF(OR(G18="",H18=""),"",IF(G18=0,IF(H18=0,0,1),I18/G18))</x:f>
+        <x:f>IF(ISNUMBER(I18),IF(G18=0,"N/A",I18/G18),"")</x:f>
       </x:c>
       <x:c r="K18" s="57" t="str"/>
       <x:c r="L18" s="57" t="str">
-        <x:f>IF(OR(I18="",K18=""),"",I18*K18)</x:f>
+        <x:f>IF(AND(ISNUMBER(I18),ISNUMBER(K18),K18&gt;=0),I18*K18,"")</x:f>
       </x:c>
       <x:c r="M18" s="42" t="str">
-        <x:f>IF(I18="","",IF(I18=0,"MATCHED",IF(I18&lt;0,"SHORTAGE","EXCESS")))</x:f>
+        <x:f>IF(COUNTA(B18:H18,K18)=0,"",IF(ISNUMBER(I18),IF(I18=0,"MATCHED",IF(I18&lt;0,"SHORTAGE","EXCESS")),"INCOMPLETE"))</x:f>
       </x:c>
     </x:row>
     <x:row r="19">
@@ -877,17 +917,17 @@
       <x:c r="G19" s="48" t="str"/>
       <x:c r="H19" s="48" t="str"/>
       <x:c r="I19" s="48" t="str">
-        <x:f>IF(OR(G19="",H19=""),"",H19-G19)</x:f>
+        <x:f>IF(AND(ISNUMBER(G19),ISNUMBER(H19),G19&gt;=0,H19&gt;=0),H19-G19,"")</x:f>
       </x:c>
       <x:c r="J19" s="52" t="str">
-        <x:f>IF(OR(G19="",H19=""),"",IF(G19=0,IF(H19=0,0,1),I19/G19))</x:f>
+        <x:f>IF(ISNUMBER(I19),IF(G19=0,"N/A",I19/G19),"")</x:f>
       </x:c>
       <x:c r="K19" s="56" t="str"/>
       <x:c r="L19" s="56" t="str">
-        <x:f>IF(OR(I19="",K19=""),"",I19*K19)</x:f>
+        <x:f>IF(AND(ISNUMBER(I19),ISNUMBER(K19),K19&gt;=0),I19*K19,"")</x:f>
       </x:c>
       <x:c r="M19" s="40" t="str">
-        <x:f>IF(I19="","",IF(I19=0,"MATCHED",IF(I19&lt;0,"SHORTAGE","EXCESS")))</x:f>
+        <x:f>IF(COUNTA(B19:H19,K19)=0,"",IF(ISNUMBER(I19),IF(I19=0,"MATCHED",IF(I19&lt;0,"SHORTAGE","EXCESS")),"INCOMPLETE"))</x:f>
       </x:c>
     </x:row>
     <x:row r="20">
@@ -902,17 +942,17 @@
       <x:c r="G20" s="49" t="str"/>
       <x:c r="H20" s="49" t="str"/>
       <x:c r="I20" s="49" t="str">
-        <x:f>IF(OR(G20="",H20=""),"",H20-G20)</x:f>
+        <x:f>IF(AND(ISNUMBER(G20),ISNUMBER(H20),G20&gt;=0,H20&gt;=0),H20-G20,"")</x:f>
       </x:c>
       <x:c r="J20" s="53" t="str">
-        <x:f>IF(OR(G20="",H20=""),"",IF(G20=0,IF(H20=0,0,1),I20/G20))</x:f>
+        <x:f>IF(ISNUMBER(I20),IF(G20=0,"N/A",I20/G20),"")</x:f>
       </x:c>
       <x:c r="K20" s="57" t="str"/>
       <x:c r="L20" s="57" t="str">
-        <x:f>IF(OR(I20="",K20=""),"",I20*K20)</x:f>
+        <x:f>IF(AND(ISNUMBER(I20),ISNUMBER(K20),K20&gt;=0),I20*K20,"")</x:f>
       </x:c>
       <x:c r="M20" s="42" t="str">
-        <x:f>IF(I20="","",IF(I20=0,"MATCHED",IF(I20&lt;0,"SHORTAGE","EXCESS")))</x:f>
+        <x:f>IF(COUNTA(B20:H20,K20)=0,"",IF(ISNUMBER(I20),IF(I20=0,"MATCHED",IF(I20&lt;0,"SHORTAGE","EXCESS")),"INCOMPLETE"))</x:f>
       </x:c>
     </x:row>
     <x:row r="21">
@@ -927,17 +967,17 @@
       <x:c r="G21" s="48" t="str"/>
       <x:c r="H21" s="48" t="str"/>
       <x:c r="I21" s="48" t="str">
-        <x:f>IF(OR(G21="",H21=""),"",H21-G21)</x:f>
+        <x:f>IF(AND(ISNUMBER(G21),ISNUMBER(H21),G21&gt;=0,H21&gt;=0),H21-G21,"")</x:f>
       </x:c>
       <x:c r="J21" s="52" t="str">
-        <x:f>IF(OR(G21="",H21=""),"",IF(G21=0,IF(H21=0,0,1),I21/G21))</x:f>
+        <x:f>IF(ISNUMBER(I21),IF(G21=0,"N/A",I21/G21),"")</x:f>
       </x:c>
       <x:c r="K21" s="56" t="str"/>
       <x:c r="L21" s="56" t="str">
-        <x:f>IF(OR(I21="",K21=""),"",I21*K21)</x:f>
+        <x:f>IF(AND(ISNUMBER(I21),ISNUMBER(K21),K21&gt;=0),I21*K21,"")</x:f>
       </x:c>
       <x:c r="M21" s="40" t="str">
-        <x:f>IF(I21="","",IF(I21=0,"MATCHED",IF(I21&lt;0,"SHORTAGE","EXCESS")))</x:f>
+        <x:f>IF(COUNTA(B21:H21,K21)=0,"",IF(ISNUMBER(I21),IF(I21=0,"MATCHED",IF(I21&lt;0,"SHORTAGE","EXCESS")),"INCOMPLETE"))</x:f>
       </x:c>
     </x:row>
     <x:row r="22">
@@ -952,17 +992,17 @@
       <x:c r="G22" s="49" t="str"/>
       <x:c r="H22" s="49" t="str"/>
       <x:c r="I22" s="49" t="str">
-        <x:f>IF(OR(G22="",H22=""),"",H22-G22)</x:f>
+        <x:f>IF(AND(ISNUMBER(G22),ISNUMBER(H22),G22&gt;=0,H22&gt;=0),H22-G22,"")</x:f>
       </x:c>
       <x:c r="J22" s="53" t="str">
-        <x:f>IF(OR(G22="",H22=""),"",IF(G22=0,IF(H22=0,0,1),I22/G22))</x:f>
+        <x:f>IF(ISNUMBER(I22),IF(G22=0,"N/A",I22/G22),"")</x:f>
       </x:c>
       <x:c r="K22" s="57" t="str"/>
       <x:c r="L22" s="57" t="str">
-        <x:f>IF(OR(I22="",K22=""),"",I22*K22)</x:f>
+        <x:f>IF(AND(ISNUMBER(I22),ISNUMBER(K22),K22&gt;=0),I22*K22,"")</x:f>
       </x:c>
       <x:c r="M22" s="42" t="str">
-        <x:f>IF(I22="","",IF(I22=0,"MATCHED",IF(I22&lt;0,"SHORTAGE","EXCESS")))</x:f>
+        <x:f>IF(COUNTA(B22:H22,K22)=0,"",IF(ISNUMBER(I22),IF(I22=0,"MATCHED",IF(I22&lt;0,"SHORTAGE","EXCESS")),"INCOMPLETE"))</x:f>
       </x:c>
     </x:row>
     <x:row r="23">
@@ -977,17 +1017,17 @@
       <x:c r="G23" s="48" t="str"/>
       <x:c r="H23" s="48" t="str"/>
       <x:c r="I23" s="48" t="str">
-        <x:f>IF(OR(G23="",H23=""),"",H23-G23)</x:f>
+        <x:f>IF(AND(ISNUMBER(G23),ISNUMBER(H23),G23&gt;=0,H23&gt;=0),H23-G23,"")</x:f>
       </x:c>
       <x:c r="J23" s="52" t="str">
-        <x:f>IF(OR(G23="",H23=""),"",IF(G23=0,IF(H23=0,0,1),I23/G23))</x:f>
+        <x:f>IF(ISNUMBER(I23),IF(G23=0,"N/A",I23/G23),"")</x:f>
       </x:c>
       <x:c r="K23" s="56" t="str"/>
       <x:c r="L23" s="56" t="str">
-        <x:f>IF(OR(I23="",K23=""),"",I23*K23)</x:f>
+        <x:f>IF(AND(ISNUMBER(I23),ISNUMBER(K23),K23&gt;=0),I23*K23,"")</x:f>
       </x:c>
       <x:c r="M23" s="40" t="str">
-        <x:f>IF(I23="","",IF(I23=0,"MATCHED",IF(I23&lt;0,"SHORTAGE","EXCESS")))</x:f>
+        <x:f>IF(COUNTA(B23:H23,K23)=0,"",IF(ISNUMBER(I23),IF(I23=0,"MATCHED",IF(I23&lt;0,"SHORTAGE","EXCESS")),"INCOMPLETE"))</x:f>
       </x:c>
     </x:row>
     <x:row r="24">
@@ -1002,17 +1042,17 @@
       <x:c r="G24" s="49" t="str"/>
       <x:c r="H24" s="49" t="str"/>
       <x:c r="I24" s="49" t="str">
-        <x:f>IF(OR(G24="",H24=""),"",H24-G24)</x:f>
+        <x:f>IF(AND(ISNUMBER(G24),ISNUMBER(H24),G24&gt;=0,H24&gt;=0),H24-G24,"")</x:f>
       </x:c>
       <x:c r="J24" s="53" t="str">
-        <x:f>IF(OR(G24="",H24=""),"",IF(G24=0,IF(H24=0,0,1),I24/G24))</x:f>
+        <x:f>IF(ISNUMBER(I24),IF(G24=0,"N/A",I24/G24),"")</x:f>
       </x:c>
       <x:c r="K24" s="57" t="str"/>
       <x:c r="L24" s="57" t="str">
-        <x:f>IF(OR(I24="",K24=""),"",I24*K24)</x:f>
+        <x:f>IF(AND(ISNUMBER(I24),ISNUMBER(K24),K24&gt;=0),I24*K24,"")</x:f>
       </x:c>
       <x:c r="M24" s="42" t="str">
-        <x:f>IF(I24="","",IF(I24=0,"MATCHED",IF(I24&lt;0,"SHORTAGE","EXCESS")))</x:f>
+        <x:f>IF(COUNTA(B24:H24,K24)=0,"",IF(ISNUMBER(I24),IF(I24=0,"MATCHED",IF(I24&lt;0,"SHORTAGE","EXCESS")),"INCOMPLETE"))</x:f>
       </x:c>
     </x:row>
     <x:row r="25">
@@ -1027,17 +1067,17 @@
       <x:c r="G25" s="48" t="str"/>
       <x:c r="H25" s="48" t="str"/>
       <x:c r="I25" s="48" t="str">
-        <x:f>IF(OR(G25="",H25=""),"",H25-G25)</x:f>
+        <x:f>IF(AND(ISNUMBER(G25),ISNUMBER(H25),G25&gt;=0,H25&gt;=0),H25-G25,"")</x:f>
       </x:c>
       <x:c r="J25" s="52" t="str">
-        <x:f>IF(OR(G25="",H25=""),"",IF(G25=0,IF(H25=0,0,1),I25/G25))</x:f>
+        <x:f>IF(ISNUMBER(I25),IF(G25=0,"N/A",I25/G25),"")</x:f>
       </x:c>
       <x:c r="K25" s="56" t="str"/>
       <x:c r="L25" s="56" t="str">
-        <x:f>IF(OR(I25="",K25=""),"",I25*K25)</x:f>
+        <x:f>IF(AND(ISNUMBER(I25),ISNUMBER(K25),K25&gt;=0),I25*K25,"")</x:f>
       </x:c>
       <x:c r="M25" s="40" t="str">
-        <x:f>IF(I25="","",IF(I25=0,"MATCHED",IF(I25&lt;0,"SHORTAGE","EXCESS")))</x:f>
+        <x:f>IF(COUNTA(B25:H25,K25)=0,"",IF(ISNUMBER(I25),IF(I25=0,"MATCHED",IF(I25&lt;0,"SHORTAGE","EXCESS")),"INCOMPLETE"))</x:f>
       </x:c>
     </x:row>
     <x:row r="26">
@@ -1052,17 +1092,17 @@
       <x:c r="G26" s="49" t="str"/>
       <x:c r="H26" s="49" t="str"/>
       <x:c r="I26" s="49" t="str">
-        <x:f>IF(OR(G26="",H26=""),"",H26-G26)</x:f>
+        <x:f>IF(AND(ISNUMBER(G26),ISNUMBER(H26),G26&gt;=0,H26&gt;=0),H26-G26,"")</x:f>
       </x:c>
       <x:c r="J26" s="53" t="str">
-        <x:f>IF(OR(G26="",H26=""),"",IF(G26=0,IF(H26=0,0,1),I26/G26))</x:f>
+        <x:f>IF(ISNUMBER(I26),IF(G26=0,"N/A",I26/G26),"")</x:f>
       </x:c>
       <x:c r="K26" s="57" t="str"/>
       <x:c r="L26" s="57" t="str">
-        <x:f>IF(OR(I26="",K26=""),"",I26*K26)</x:f>
+        <x:f>IF(AND(ISNUMBER(I26),ISNUMBER(K26),K26&gt;=0),I26*K26,"")</x:f>
       </x:c>
       <x:c r="M26" s="42" t="str">
-        <x:f>IF(I26="","",IF(I26=0,"MATCHED",IF(I26&lt;0,"SHORTAGE","EXCESS")))</x:f>
+        <x:f>IF(COUNTA(B26:H26,K26)=0,"",IF(ISNUMBER(I26),IF(I26=0,"MATCHED",IF(I26&lt;0,"SHORTAGE","EXCESS")),"INCOMPLETE"))</x:f>
       </x:c>
     </x:row>
     <x:row r="27">
@@ -1077,17 +1117,17 @@
       <x:c r="G27" s="48" t="str"/>
       <x:c r="H27" s="48" t="str"/>
       <x:c r="I27" s="48" t="str">
-        <x:f>IF(OR(G27="",H27=""),"",H27-G27)</x:f>
+        <x:f>IF(AND(ISNUMBER(G27),ISNUMBER(H27),G27&gt;=0,H27&gt;=0),H27-G27,"")</x:f>
       </x:c>
       <x:c r="J27" s="52" t="str">
-        <x:f>IF(OR(G27="",H27=""),"",IF(G27=0,IF(H27=0,0,1),I27/G27))</x:f>
+        <x:f>IF(ISNUMBER(I27),IF(G27=0,"N/A",I27/G27),"")</x:f>
       </x:c>
       <x:c r="K27" s="56" t="str"/>
       <x:c r="L27" s="56" t="str">
-        <x:f>IF(OR(I27="",K27=""),"",I27*K27)</x:f>
+        <x:f>IF(AND(ISNUMBER(I27),ISNUMBER(K27),K27&gt;=0),I27*K27,"")</x:f>
       </x:c>
       <x:c r="M27" s="40" t="str">
-        <x:f>IF(I27="","",IF(I27=0,"MATCHED",IF(I27&lt;0,"SHORTAGE","EXCESS")))</x:f>
+        <x:f>IF(COUNTA(B27:H27,K27)=0,"",IF(ISNUMBER(I27),IF(I27=0,"MATCHED",IF(I27&lt;0,"SHORTAGE","EXCESS")),"INCOMPLETE"))</x:f>
       </x:c>
     </x:row>
     <x:row r="28">
@@ -1102,17 +1142,17 @@
       <x:c r="G28" s="49" t="str"/>
       <x:c r="H28" s="49" t="str"/>
       <x:c r="I28" s="49" t="str">
-        <x:f>IF(OR(G28="",H28=""),"",H28-G28)</x:f>
+        <x:f>IF(AND(ISNUMBER(G28),ISNUMBER(H28),G28&gt;=0,H28&gt;=0),H28-G28,"")</x:f>
       </x:c>
       <x:c r="J28" s="53" t="str">
-        <x:f>IF(OR(G28="",H28=""),"",IF(G28=0,IF(H28=0,0,1),I28/G28))</x:f>
+        <x:f>IF(ISNUMBER(I28),IF(G28=0,"N/A",I28/G28),"")</x:f>
       </x:c>
       <x:c r="K28" s="57" t="str"/>
       <x:c r="L28" s="57" t="str">
-        <x:f>IF(OR(I28="",K28=""),"",I28*K28)</x:f>
+        <x:f>IF(AND(ISNUMBER(I28),ISNUMBER(K28),K28&gt;=0),I28*K28,"")</x:f>
       </x:c>
       <x:c r="M28" s="42" t="str">
-        <x:f>IF(I28="","",IF(I28=0,"MATCHED",IF(I28&lt;0,"SHORTAGE","EXCESS")))</x:f>
+        <x:f>IF(COUNTA(B28:H28,K28)=0,"",IF(ISNUMBER(I28),IF(I28=0,"MATCHED",IF(I28&lt;0,"SHORTAGE","EXCESS")),"INCOMPLETE"))</x:f>
       </x:c>
     </x:row>
     <x:row r="29">
@@ -1127,17 +1167,17 @@
       <x:c r="G29" s="48" t="str"/>
       <x:c r="H29" s="48" t="str"/>
       <x:c r="I29" s="48" t="str">
-        <x:f>IF(OR(G29="",H29=""),"",H29-G29)</x:f>
+        <x:f>IF(AND(ISNUMBER(G29),ISNUMBER(H29),G29&gt;=0,H29&gt;=0),H29-G29,"")</x:f>
       </x:c>
       <x:c r="J29" s="52" t="str">
-        <x:f>IF(OR(G29="",H29=""),"",IF(G29=0,IF(H29=0,0,1),I29/G29))</x:f>
+        <x:f>IF(ISNUMBER(I29),IF(G29=0,"N/A",I29/G29),"")</x:f>
       </x:c>
       <x:c r="K29" s="56" t="str"/>
       <x:c r="L29" s="56" t="str">
-        <x:f>IF(OR(I29="",K29=""),"",I29*K29)</x:f>
+        <x:f>IF(AND(ISNUMBER(I29),ISNUMBER(K29),K29&gt;=0),I29*K29,"")</x:f>
       </x:c>
       <x:c r="M29" s="40" t="str">
-        <x:f>IF(I29="","",IF(I29=0,"MATCHED",IF(I29&lt;0,"SHORTAGE","EXCESS")))</x:f>
+        <x:f>IF(COUNTA(B29:H29,K29)=0,"",IF(ISNUMBER(I29),IF(I29=0,"MATCHED",IF(I29&lt;0,"SHORTAGE","EXCESS")),"INCOMPLETE"))</x:f>
       </x:c>
     </x:row>
     <x:row r="30">
@@ -1152,17 +1192,17 @@
       <x:c r="G30" s="49" t="str"/>
       <x:c r="H30" s="49" t="str"/>
       <x:c r="I30" s="49" t="str">
-        <x:f>IF(OR(G30="",H30=""),"",H30-G30)</x:f>
+        <x:f>IF(AND(ISNUMBER(G30),ISNUMBER(H30),G30&gt;=0,H30&gt;=0),H30-G30,"")</x:f>
       </x:c>
       <x:c r="J30" s="53" t="str">
-        <x:f>IF(OR(G30="",H30=""),"",IF(G30=0,IF(H30=0,0,1),I30/G30))</x:f>
+        <x:f>IF(ISNUMBER(I30),IF(G30=0,"N/A",I30/G30),"")</x:f>
       </x:c>
       <x:c r="K30" s="57" t="str"/>
       <x:c r="L30" s="57" t="str">
-        <x:f>IF(OR(I30="",K30=""),"",I30*K30)</x:f>
+        <x:f>IF(AND(ISNUMBER(I30),ISNUMBER(K30),K30&gt;=0),I30*K30,"")</x:f>
       </x:c>
       <x:c r="M30" s="42" t="str">
-        <x:f>IF(I30="","",IF(I30=0,"MATCHED",IF(I30&lt;0,"SHORTAGE","EXCESS")))</x:f>
+        <x:f>IF(COUNTA(B30:H30,K30)=0,"",IF(ISNUMBER(I30),IF(I30=0,"MATCHED",IF(I30&lt;0,"SHORTAGE","EXCESS")),"INCOMPLETE"))</x:f>
       </x:c>
     </x:row>
     <x:row r="31">
@@ -1177,17 +1217,17 @@
       <x:c r="G31" s="48" t="str"/>
       <x:c r="H31" s="48" t="str"/>
       <x:c r="I31" s="48" t="str">
-        <x:f>IF(OR(G31="",H31=""),"",H31-G31)</x:f>
+        <x:f>IF(AND(ISNUMBER(G31),ISNUMBER(H31),G31&gt;=0,H31&gt;=0),H31-G31,"")</x:f>
       </x:c>
       <x:c r="J31" s="52" t="str">
-        <x:f>IF(OR(G31="",H31=""),"",IF(G31=0,IF(H31=0,0,1),I31/G31))</x:f>
+        <x:f>IF(ISNUMBER(I31),IF(G31=0,"N/A",I31/G31),"")</x:f>
       </x:c>
       <x:c r="K31" s="56" t="str"/>
       <x:c r="L31" s="56" t="str">
-        <x:f>IF(OR(I31="",K31=""),"",I31*K31)</x:f>
+        <x:f>IF(AND(ISNUMBER(I31),ISNUMBER(K31),K31&gt;=0),I31*K31,"")</x:f>
       </x:c>
       <x:c r="M31" s="40" t="str">
-        <x:f>IF(I31="","",IF(I31=0,"MATCHED",IF(I31&lt;0,"SHORTAGE","EXCESS")))</x:f>
+        <x:f>IF(COUNTA(B31:H31,K31)=0,"",IF(ISNUMBER(I31),IF(I31=0,"MATCHED",IF(I31&lt;0,"SHORTAGE","EXCESS")),"INCOMPLETE"))</x:f>
       </x:c>
     </x:row>
     <x:row r="32">
@@ -1202,17 +1242,17 @@
       <x:c r="G32" s="49" t="str"/>
       <x:c r="H32" s="49" t="str"/>
       <x:c r="I32" s="49" t="str">
-        <x:f>IF(OR(G32="",H32=""),"",H32-G32)</x:f>
+        <x:f>IF(AND(ISNUMBER(G32),ISNUMBER(H32),G32&gt;=0,H32&gt;=0),H32-G32,"")</x:f>
       </x:c>
       <x:c r="J32" s="53" t="str">
-        <x:f>IF(OR(G32="",H32=""),"",IF(G32=0,IF(H32=0,0,1),I32/G32))</x:f>
+        <x:f>IF(ISNUMBER(I32),IF(G32=0,"N/A",I32/G32),"")</x:f>
       </x:c>
       <x:c r="K32" s="57" t="str"/>
       <x:c r="L32" s="57" t="str">
-        <x:f>IF(OR(I32="",K32=""),"",I32*K32)</x:f>
+        <x:f>IF(AND(ISNUMBER(I32),ISNUMBER(K32),K32&gt;=0),I32*K32,"")</x:f>
       </x:c>
       <x:c r="M32" s="42" t="str">
-        <x:f>IF(I32="","",IF(I32=0,"MATCHED",IF(I32&lt;0,"SHORTAGE","EXCESS")))</x:f>
+        <x:f>IF(COUNTA(B32:H32,K32)=0,"",IF(ISNUMBER(I32),IF(I32=0,"MATCHED",IF(I32&lt;0,"SHORTAGE","EXCESS")),"INCOMPLETE"))</x:f>
       </x:c>
     </x:row>
     <x:row r="33">
@@ -1227,17 +1267,17 @@
       <x:c r="G33" s="48" t="str"/>
       <x:c r="H33" s="48" t="str"/>
       <x:c r="I33" s="48" t="str">
-        <x:f>IF(OR(G33="",H33=""),"",H33-G33)</x:f>
+        <x:f>IF(AND(ISNUMBER(G33),ISNUMBER(H33),G33&gt;=0,H33&gt;=0),H33-G33,"")</x:f>
       </x:c>
       <x:c r="J33" s="52" t="str">
-        <x:f>IF(OR(G33="",H33=""),"",IF(G33=0,IF(H33=0,0,1),I33/G33))</x:f>
+        <x:f>IF(ISNUMBER(I33),IF(G33=0,"N/A",I33/G33),"")</x:f>
       </x:c>
       <x:c r="K33" s="56" t="str"/>
       <x:c r="L33" s="56" t="str">
-        <x:f>IF(OR(I33="",K33=""),"",I33*K33)</x:f>
+        <x:f>IF(AND(ISNUMBER(I33),ISNUMBER(K33),K33&gt;=0),I33*K33,"")</x:f>
       </x:c>
       <x:c r="M33" s="40" t="str">
-        <x:f>IF(I33="","",IF(I33=0,"MATCHED",IF(I33&lt;0,"SHORTAGE","EXCESS")))</x:f>
+        <x:f>IF(COUNTA(B33:H33,K33)=0,"",IF(ISNUMBER(I33),IF(I33=0,"MATCHED",IF(I33&lt;0,"SHORTAGE","EXCESS")),"INCOMPLETE"))</x:f>
       </x:c>
     </x:row>
     <x:row r="34">
@@ -1252,17 +1292,17 @@
       <x:c r="G34" s="49" t="str"/>
       <x:c r="H34" s="49" t="str"/>
       <x:c r="I34" s="49" t="str">
-        <x:f>IF(OR(G34="",H34=""),"",H34-G34)</x:f>
+        <x:f>IF(AND(ISNUMBER(G34),ISNUMBER(H34),G34&gt;=0,H34&gt;=0),H34-G34,"")</x:f>
       </x:c>
       <x:c r="J34" s="53" t="str">
-        <x:f>IF(OR(G34="",H34=""),"",IF(G34=0,IF(H34=0,0,1),I34/G34))</x:f>
+        <x:f>IF(ISNUMBER(I34),IF(G34=0,"N/A",I34/G34),"")</x:f>
       </x:c>
       <x:c r="K34" s="57" t="str"/>
       <x:c r="L34" s="57" t="str">
-        <x:f>IF(OR(I34="",K34=""),"",I34*K34)</x:f>
+        <x:f>IF(AND(ISNUMBER(I34),ISNUMBER(K34),K34&gt;=0),I34*K34,"")</x:f>
       </x:c>
       <x:c r="M34" s="42" t="str">
-        <x:f>IF(I34="","",IF(I34=0,"MATCHED",IF(I34&lt;0,"SHORTAGE","EXCESS")))</x:f>
+        <x:f>IF(COUNTA(B34:H34,K34)=0,"",IF(ISNUMBER(I34),IF(I34=0,"MATCHED",IF(I34&lt;0,"SHORTAGE","EXCESS")),"INCOMPLETE"))</x:f>
       </x:c>
     </x:row>
     <x:row r="35">
@@ -1277,17 +1317,17 @@
       <x:c r="G35" s="48" t="str"/>
       <x:c r="H35" s="48" t="str"/>
       <x:c r="I35" s="48" t="str">
-        <x:f>IF(OR(G35="",H35=""),"",H35-G35)</x:f>
+        <x:f>IF(AND(ISNUMBER(G35),ISNUMBER(H35),G35&gt;=0,H35&gt;=0),H35-G35,"")</x:f>
       </x:c>
       <x:c r="J35" s="52" t="str">
-        <x:f>IF(OR(G35="",H35=""),"",IF(G35=0,IF(H35=0,0,1),I35/G35))</x:f>
+        <x:f>IF(ISNUMBER(I35),IF(G35=0,"N/A",I35/G35),"")</x:f>
       </x:c>
       <x:c r="K35" s="56" t="str"/>
       <x:c r="L35" s="56" t="str">
-        <x:f>IF(OR(I35="",K35=""),"",I35*K35)</x:f>
+        <x:f>IF(AND(ISNUMBER(I35),ISNUMBER(K35),K35&gt;=0),I35*K35,"")</x:f>
       </x:c>
       <x:c r="M35" s="40" t="str">
-        <x:f>IF(I35="","",IF(I35=0,"MATCHED",IF(I35&lt;0,"SHORTAGE","EXCESS")))</x:f>
+        <x:f>IF(COUNTA(B35:H35,K35)=0,"",IF(ISNUMBER(I35),IF(I35=0,"MATCHED",IF(I35&lt;0,"SHORTAGE","EXCESS")),"INCOMPLETE"))</x:f>
       </x:c>
     </x:row>
     <x:row r="36">
@@ -1302,17 +1342,17 @@
       <x:c r="G36" s="49" t="str"/>
       <x:c r="H36" s="49" t="str"/>
       <x:c r="I36" s="49" t="str">
-        <x:f>IF(OR(G36="",H36=""),"",H36-G36)</x:f>
+        <x:f>IF(AND(ISNUMBER(G36),ISNUMBER(H36),G36&gt;=0,H36&gt;=0),H36-G36,"")</x:f>
       </x:c>
       <x:c r="J36" s="53" t="str">
-        <x:f>IF(OR(G36="",H36=""),"",IF(G36=0,IF(H36=0,0,1),I36/G36))</x:f>
+        <x:f>IF(ISNUMBER(I36),IF(G36=0,"N/A",I36/G36),"")</x:f>
       </x:c>
       <x:c r="K36" s="57" t="str"/>
       <x:c r="L36" s="57" t="str">
-        <x:f>IF(OR(I36="",K36=""),"",I36*K36)</x:f>
+        <x:f>IF(AND(ISNUMBER(I36),ISNUMBER(K36),K36&gt;=0),I36*K36,"")</x:f>
       </x:c>
       <x:c r="M36" s="42" t="str">
-        <x:f>IF(I36="","",IF(I36=0,"MATCHED",IF(I36&lt;0,"SHORTAGE","EXCESS")))</x:f>
+        <x:f>IF(COUNTA(B36:H36,K36)=0,"",IF(ISNUMBER(I36),IF(I36=0,"MATCHED",IF(I36&lt;0,"SHORTAGE","EXCESS")),"INCOMPLETE"))</x:f>
       </x:c>
     </x:row>
     <x:row r="37">
@@ -1327,17 +1367,17 @@
       <x:c r="G37" s="48" t="str"/>
       <x:c r="H37" s="48" t="str"/>
       <x:c r="I37" s="48" t="str">
-        <x:f>IF(OR(G37="",H37=""),"",H37-G37)</x:f>
+        <x:f>IF(AND(ISNUMBER(G37),ISNUMBER(H37),G37&gt;=0,H37&gt;=0),H37-G37,"")</x:f>
       </x:c>
       <x:c r="J37" s="52" t="str">
-        <x:f>IF(OR(G37="",H37=""),"",IF(G37=0,IF(H37=0,0,1),I37/G37))</x:f>
+        <x:f>IF(ISNUMBER(I37),IF(G37=0,"N/A",I37/G37),"")</x:f>
       </x:c>
       <x:c r="K37" s="56" t="str"/>
       <x:c r="L37" s="56" t="str">
-        <x:f>IF(OR(I37="",K37=""),"",I37*K37)</x:f>
+        <x:f>IF(AND(ISNUMBER(I37),ISNUMBER(K37),K37&gt;=0),I37*K37,"")</x:f>
       </x:c>
       <x:c r="M37" s="40" t="str">
-        <x:f>IF(I37="","",IF(I37=0,"MATCHED",IF(I37&lt;0,"SHORTAGE","EXCESS")))</x:f>
+        <x:f>IF(COUNTA(B37:H37,K37)=0,"",IF(ISNUMBER(I37),IF(I37=0,"MATCHED",IF(I37&lt;0,"SHORTAGE","EXCESS")),"INCOMPLETE"))</x:f>
       </x:c>
     </x:row>
     <x:row r="38">
@@ -1352,17 +1392,17 @@
       <x:c r="G38" s="49" t="str"/>
       <x:c r="H38" s="49" t="str"/>
       <x:c r="I38" s="49" t="str">
-        <x:f>IF(OR(G38="",H38=""),"",H38-G38)</x:f>
+        <x:f>IF(AND(ISNUMBER(G38),ISNUMBER(H38),G38&gt;=0,H38&gt;=0),H38-G38,"")</x:f>
       </x:c>
       <x:c r="J38" s="53" t="str">
-        <x:f>IF(OR(G38="",H38=""),"",IF(G38=0,IF(H38=0,0,1),I38/G38))</x:f>
+        <x:f>IF(ISNUMBER(I38),IF(G38=0,"N/A",I38/G38),"")</x:f>
       </x:c>
       <x:c r="K38" s="57" t="str"/>
       <x:c r="L38" s="57" t="str">
-        <x:f>IF(OR(I38="",K38=""),"",I38*K38)</x:f>
+        <x:f>IF(AND(ISNUMBER(I38),ISNUMBER(K38),K38&gt;=0),I38*K38,"")</x:f>
       </x:c>
       <x:c r="M38" s="42" t="str">
-        <x:f>IF(I38="","",IF(I38=0,"MATCHED",IF(I38&lt;0,"SHORTAGE","EXCESS")))</x:f>
+        <x:f>IF(COUNTA(B38:H38,K38)=0,"",IF(ISNUMBER(I38),IF(I38=0,"MATCHED",IF(I38&lt;0,"SHORTAGE","EXCESS")),"INCOMPLETE"))</x:f>
       </x:c>
     </x:row>
     <x:row r="39">
@@ -1377,17 +1417,17 @@
       <x:c r="G39" s="48" t="str"/>
       <x:c r="H39" s="48" t="str"/>
       <x:c r="I39" s="48" t="str">
-        <x:f>IF(OR(G39="",H39=""),"",H39-G39)</x:f>
+        <x:f>IF(AND(ISNUMBER(G39),ISNUMBER(H39),G39&gt;=0,H39&gt;=0),H39-G39,"")</x:f>
       </x:c>
       <x:c r="J39" s="52" t="str">
-        <x:f>IF(OR(G39="",H39=""),"",IF(G39=0,IF(H39=0,0,1),I39/G39))</x:f>
+        <x:f>IF(ISNUMBER(I39),IF(G39=0,"N/A",I39/G39),"")</x:f>
       </x:c>
       <x:c r="K39" s="56" t="str"/>
       <x:c r="L39" s="56" t="str">
-        <x:f>IF(OR(I39="",K39=""),"",I39*K39)</x:f>
+        <x:f>IF(AND(ISNUMBER(I39),ISNUMBER(K39),K39&gt;=0),I39*K39,"")</x:f>
       </x:c>
       <x:c r="M39" s="40" t="str">
-        <x:f>IF(I39="","",IF(I39=0,"MATCHED",IF(I39&lt;0,"SHORTAGE","EXCESS")))</x:f>
+        <x:f>IF(COUNTA(B39:H39,K39)=0,"",IF(ISNUMBER(I39),IF(I39=0,"MATCHED",IF(I39&lt;0,"SHORTAGE","EXCESS")),"INCOMPLETE"))</x:f>
       </x:c>
     </x:row>
     <x:row r="40">
@@ -1402,17 +1442,17 @@
       <x:c r="G40" s="49" t="str"/>
       <x:c r="H40" s="49" t="str"/>
       <x:c r="I40" s="49" t="str">
-        <x:f>IF(OR(G40="",H40=""),"",H40-G40)</x:f>
+        <x:f>IF(AND(ISNUMBER(G40),ISNUMBER(H40),G40&gt;=0,H40&gt;=0),H40-G40,"")</x:f>
       </x:c>
       <x:c r="J40" s="53" t="str">
-        <x:f>IF(OR(G40="",H40=""),"",IF(G40=0,IF(H40=0,0,1),I40/G40))</x:f>
+        <x:f>IF(ISNUMBER(I40),IF(G40=0,"N/A",I40/G40),"")</x:f>
       </x:c>
       <x:c r="K40" s="57" t="str"/>
       <x:c r="L40" s="57" t="str">
-        <x:f>IF(OR(I40="",K40=""),"",I40*K40)</x:f>
+        <x:f>IF(AND(ISNUMBER(I40),ISNUMBER(K40),K40&gt;=0),I40*K40,"")</x:f>
       </x:c>
       <x:c r="M40" s="42" t="str">
-        <x:f>IF(I40="","",IF(I40=0,"MATCHED",IF(I40&lt;0,"SHORTAGE","EXCESS")))</x:f>
+        <x:f>IF(COUNTA(B40:H40,K40)=0,"",IF(ISNUMBER(I40),IF(I40=0,"MATCHED",IF(I40&lt;0,"SHORTAGE","EXCESS")),"INCOMPLETE"))</x:f>
       </x:c>
     </x:row>
     <x:row r="41">
@@ -1427,17 +1467,17 @@
       <x:c r="G41" s="48" t="str"/>
       <x:c r="H41" s="48" t="str"/>
       <x:c r="I41" s="48" t="str">
-        <x:f>IF(OR(G41="",H41=""),"",H41-G41)</x:f>
+        <x:f>IF(AND(ISNUMBER(G41),ISNUMBER(H41),G41&gt;=0,H41&gt;=0),H41-G41,"")</x:f>
       </x:c>
       <x:c r="J41" s="52" t="str">
-        <x:f>IF(OR(G41="",H41=""),"",IF(G41=0,IF(H41=0,0,1),I41/G41))</x:f>
+        <x:f>IF(ISNUMBER(I41),IF(G41=0,"N/A",I41/G41),"")</x:f>
       </x:c>
       <x:c r="K41" s="56" t="str"/>
       <x:c r="L41" s="56" t="str">
-        <x:f>IF(OR(I41="",K41=""),"",I41*K41)</x:f>
+        <x:f>IF(AND(ISNUMBER(I41),ISNUMBER(K41),K41&gt;=0),I41*K41,"")</x:f>
       </x:c>
       <x:c r="M41" s="40" t="str">
-        <x:f>IF(I41="","",IF(I41=0,"MATCHED",IF(I41&lt;0,"SHORTAGE","EXCESS")))</x:f>
+        <x:f>IF(COUNTA(B41:H41,K41)=0,"",IF(ISNUMBER(I41),IF(I41=0,"MATCHED",IF(I41&lt;0,"SHORTAGE","EXCESS")),"INCOMPLETE"))</x:f>
       </x:c>
     </x:row>
     <x:row r="42">
@@ -1452,17 +1492,17 @@
       <x:c r="G42" s="49" t="str"/>
       <x:c r="H42" s="49" t="str"/>
       <x:c r="I42" s="49" t="str">
-        <x:f>IF(OR(G42="",H42=""),"",H42-G42)</x:f>
+        <x:f>IF(AND(ISNUMBER(G42),ISNUMBER(H42),G42&gt;=0,H42&gt;=0),H42-G42,"")</x:f>
       </x:c>
       <x:c r="J42" s="53" t="str">
-        <x:f>IF(OR(G42="",H42=""),"",IF(G42=0,IF(H42=0,0,1),I42/G42))</x:f>
+        <x:f>IF(ISNUMBER(I42),IF(G42=0,"N/A",I42/G42),"")</x:f>
       </x:c>
       <x:c r="K42" s="57" t="str"/>
       <x:c r="L42" s="57" t="str">
-        <x:f>IF(OR(I42="",K42=""),"",I42*K42)</x:f>
+        <x:f>IF(AND(ISNUMBER(I42),ISNUMBER(K42),K42&gt;=0),I42*K42,"")</x:f>
       </x:c>
       <x:c r="M42" s="42" t="str">
-        <x:f>IF(I42="","",IF(I42=0,"MATCHED",IF(I42&lt;0,"SHORTAGE","EXCESS")))</x:f>
+        <x:f>IF(COUNTA(B42:H42,K42)=0,"",IF(ISNUMBER(I42),IF(I42=0,"MATCHED",IF(I42&lt;0,"SHORTAGE","EXCESS")),"INCOMPLETE"))</x:f>
       </x:c>
     </x:row>
     <x:row r="43">
@@ -1477,17 +1517,17 @@
       <x:c r="G43" s="48" t="str"/>
       <x:c r="H43" s="48" t="str"/>
       <x:c r="I43" s="48" t="str">
-        <x:f>IF(OR(G43="",H43=""),"",H43-G43)</x:f>
+        <x:f>IF(AND(ISNUMBER(G43),ISNUMBER(H43),G43&gt;=0,H43&gt;=0),H43-G43,"")</x:f>
       </x:c>
       <x:c r="J43" s="52" t="str">
-        <x:f>IF(OR(G43="",H43=""),"",IF(G43=0,IF(H43=0,0,1),I43/G43))</x:f>
+        <x:f>IF(ISNUMBER(I43),IF(G43=0,"N/A",I43/G43),"")</x:f>
       </x:c>
       <x:c r="K43" s="56" t="str"/>
       <x:c r="L43" s="56" t="str">
-        <x:f>IF(OR(I43="",K43=""),"",I43*K43)</x:f>
+        <x:f>IF(AND(ISNUMBER(I43),ISNUMBER(K43),K43&gt;=0),I43*K43,"")</x:f>
       </x:c>
       <x:c r="M43" s="40" t="str">
-        <x:f>IF(I43="","",IF(I43=0,"MATCHED",IF(I43&lt;0,"SHORTAGE","EXCESS")))</x:f>
+        <x:f>IF(COUNTA(B43:H43,K43)=0,"",IF(ISNUMBER(I43),IF(I43=0,"MATCHED",IF(I43&lt;0,"SHORTAGE","EXCESS")),"INCOMPLETE"))</x:f>
       </x:c>
     </x:row>
     <x:row r="44">
@@ -1502,17 +1542,17 @@
       <x:c r="G44" s="49" t="str"/>
       <x:c r="H44" s="49" t="str"/>
       <x:c r="I44" s="49" t="str">
-        <x:f>IF(OR(G44="",H44=""),"",H44-G44)</x:f>
+        <x:f>IF(AND(ISNUMBER(G44),ISNUMBER(H44),G44&gt;=0,H44&gt;=0),H44-G44,"")</x:f>
       </x:c>
       <x:c r="J44" s="53" t="str">
-        <x:f>IF(OR(G44="",H44=""),"",IF(G44=0,IF(H44=0,0,1),I44/G44))</x:f>
+        <x:f>IF(ISNUMBER(I44),IF(G44=0,"N/A",I44/G44),"")</x:f>
       </x:c>
       <x:c r="K44" s="57" t="str"/>
       <x:c r="L44" s="57" t="str">
-        <x:f>IF(OR(I44="",K44=""),"",I44*K44)</x:f>
+        <x:f>IF(AND(ISNUMBER(I44),ISNUMBER(K44),K44&gt;=0),I44*K44,"")</x:f>
       </x:c>
       <x:c r="M44" s="42" t="str">
-        <x:f>IF(I44="","",IF(I44=0,"MATCHED",IF(I44&lt;0,"SHORTAGE","EXCESS")))</x:f>
+        <x:f>IF(COUNTA(B44:H44,K44)=0,"",IF(ISNUMBER(I44),IF(I44=0,"MATCHED",IF(I44&lt;0,"SHORTAGE","EXCESS")),"INCOMPLETE"))</x:f>
       </x:c>
     </x:row>
     <x:row r="45">
@@ -1527,17 +1567,17 @@
       <x:c r="G45" s="48" t="str"/>
       <x:c r="H45" s="48" t="str"/>
       <x:c r="I45" s="48" t="str">
-        <x:f>IF(OR(G45="",H45=""),"",H45-G45)</x:f>
+        <x:f>IF(AND(ISNUMBER(G45),ISNUMBER(H45),G45&gt;=0,H45&gt;=0),H45-G45,"")</x:f>
       </x:c>
       <x:c r="J45" s="52" t="str">
-        <x:f>IF(OR(G45="",H45=""),"",IF(G45=0,IF(H45=0,0,1),I45/G45))</x:f>
+        <x:f>IF(ISNUMBER(I45),IF(G45=0,"N/A",I45/G45),"")</x:f>
       </x:c>
       <x:c r="K45" s="56" t="str"/>
       <x:c r="L45" s="56" t="str">
-        <x:f>IF(OR(I45="",K45=""),"",I45*K45)</x:f>
+        <x:f>IF(AND(ISNUMBER(I45),ISNUMBER(K45),K45&gt;=0),I45*K45,"")</x:f>
       </x:c>
       <x:c r="M45" s="40" t="str">
-        <x:f>IF(I45="","",IF(I45=0,"MATCHED",IF(I45&lt;0,"SHORTAGE","EXCESS")))</x:f>
+        <x:f>IF(COUNTA(B45:H45,K45)=0,"",IF(ISNUMBER(I45),IF(I45=0,"MATCHED",IF(I45&lt;0,"SHORTAGE","EXCESS")),"INCOMPLETE"))</x:f>
       </x:c>
     </x:row>
     <x:row r="46">
@@ -1552,17 +1592,17 @@
       <x:c r="G46" s="49" t="str"/>
       <x:c r="H46" s="49" t="str"/>
       <x:c r="I46" s="49" t="str">
-        <x:f>IF(OR(G46="",H46=""),"",H46-G46)</x:f>
+        <x:f>IF(AND(ISNUMBER(G46),ISNUMBER(H46),G46&gt;=0,H46&gt;=0),H46-G46,"")</x:f>
       </x:c>
       <x:c r="J46" s="53" t="str">
-        <x:f>IF(OR(G46="",H46=""),"",IF(G46=0,IF(H46=0,0,1),I46/G46))</x:f>
+        <x:f>IF(ISNUMBER(I46),IF(G46=0,"N/A",I46/G46),"")</x:f>
       </x:c>
       <x:c r="K46" s="57" t="str"/>
       <x:c r="L46" s="57" t="str">
-        <x:f>IF(OR(I46="",K46=""),"",I46*K46)</x:f>
+        <x:f>IF(AND(ISNUMBER(I46),ISNUMBER(K46),K46&gt;=0),I46*K46,"")</x:f>
       </x:c>
       <x:c r="M46" s="42" t="str">
-        <x:f>IF(I46="","",IF(I46=0,"MATCHED",IF(I46&lt;0,"SHORTAGE","EXCESS")))</x:f>
+        <x:f>IF(COUNTA(B46:H46,K46)=0,"",IF(ISNUMBER(I46),IF(I46=0,"MATCHED",IF(I46&lt;0,"SHORTAGE","EXCESS")),"INCOMPLETE"))</x:f>
       </x:c>
     </x:row>
     <x:row r="47">
@@ -1577,17 +1617,17 @@
       <x:c r="G47" s="48" t="str"/>
       <x:c r="H47" s="48" t="str"/>
       <x:c r="I47" s="48" t="str">
-        <x:f>IF(OR(G47="",H47=""),"",H47-G47)</x:f>
+        <x:f>IF(AND(ISNUMBER(G47),ISNUMBER(H47),G47&gt;=0,H47&gt;=0),H47-G47,"")</x:f>
       </x:c>
       <x:c r="J47" s="52" t="str">
-        <x:f>IF(OR(G47="",H47=""),"",IF(G47=0,IF(H47=0,0,1),I47/G47))</x:f>
+        <x:f>IF(ISNUMBER(I47),IF(G47=0,"N/A",I47/G47),"")</x:f>
       </x:c>
       <x:c r="K47" s="56" t="str"/>
       <x:c r="L47" s="56" t="str">
-        <x:f>IF(OR(I47="",K47=""),"",I47*K47)</x:f>
+        <x:f>IF(AND(ISNUMBER(I47),ISNUMBER(K47),K47&gt;=0),I47*K47,"")</x:f>
       </x:c>
       <x:c r="M47" s="40" t="str">
-        <x:f>IF(I47="","",IF(I47=0,"MATCHED",IF(I47&lt;0,"SHORTAGE","EXCESS")))</x:f>
+        <x:f>IF(COUNTA(B47:H47,K47)=0,"",IF(ISNUMBER(I47),IF(I47=0,"MATCHED",IF(I47&lt;0,"SHORTAGE","EXCESS")),"INCOMPLETE"))</x:f>
       </x:c>
     </x:row>
     <x:row r="48">
@@ -1602,17 +1642,17 @@
       <x:c r="G48" s="49" t="str"/>
       <x:c r="H48" s="49" t="str"/>
       <x:c r="I48" s="49" t="str">
-        <x:f>IF(OR(G48="",H48=""),"",H48-G48)</x:f>
+        <x:f>IF(AND(ISNUMBER(G48),ISNUMBER(H48),G48&gt;=0,H48&gt;=0),H48-G48,"")</x:f>
       </x:c>
       <x:c r="J48" s="53" t="str">
-        <x:f>IF(OR(G48="",H48=""),"",IF(G48=0,IF(H48=0,0,1),I48/G48))</x:f>
+        <x:f>IF(ISNUMBER(I48),IF(G48=0,"N/A",I48/G48),"")</x:f>
       </x:c>
       <x:c r="K48" s="57" t="str"/>
       <x:c r="L48" s="57" t="str">
-        <x:f>IF(OR(I48="",K48=""),"",I48*K48)</x:f>
+        <x:f>IF(AND(ISNUMBER(I48),ISNUMBER(K48),K48&gt;=0),I48*K48,"")</x:f>
       </x:c>
       <x:c r="M48" s="42" t="str">
-        <x:f>IF(I48="","",IF(I48=0,"MATCHED",IF(I48&lt;0,"SHORTAGE","EXCESS")))</x:f>
+        <x:f>IF(COUNTA(B48:H48,K48)=0,"",IF(ISNUMBER(I48),IF(I48=0,"MATCHED",IF(I48&lt;0,"SHORTAGE","EXCESS")),"INCOMPLETE"))</x:f>
       </x:c>
     </x:row>
     <x:row r="49">
@@ -1627,17 +1667,17 @@
       <x:c r="G49" s="48" t="str"/>
       <x:c r="H49" s="48" t="str"/>
       <x:c r="I49" s="48" t="str">
-        <x:f>IF(OR(G49="",H49=""),"",H49-G49)</x:f>
+        <x:f>IF(AND(ISNUMBER(G49),ISNUMBER(H49),G49&gt;=0,H49&gt;=0),H49-G49,"")</x:f>
       </x:c>
       <x:c r="J49" s="52" t="str">
-        <x:f>IF(OR(G49="",H49=""),"",IF(G49=0,IF(H49=0,0,1),I49/G49))</x:f>
+        <x:f>IF(ISNUMBER(I49),IF(G49=0,"N/A",I49/G49),"")</x:f>
       </x:c>
       <x:c r="K49" s="56" t="str"/>
       <x:c r="L49" s="56" t="str">
-        <x:f>IF(OR(I49="",K49=""),"",I49*K49)</x:f>
+        <x:f>IF(AND(ISNUMBER(I49),ISNUMBER(K49),K49&gt;=0),I49*K49,"")</x:f>
       </x:c>
       <x:c r="M49" s="40" t="str">
-        <x:f>IF(I49="","",IF(I49=0,"MATCHED",IF(I49&lt;0,"SHORTAGE","EXCESS")))</x:f>
+        <x:f>IF(COUNTA(B49:H49,K49)=0,"",IF(ISNUMBER(I49),IF(I49=0,"MATCHED",IF(I49&lt;0,"SHORTAGE","EXCESS")),"INCOMPLETE"))</x:f>
       </x:c>
     </x:row>
     <x:row r="50">
@@ -1652,17 +1692,17 @@
       <x:c r="G50" s="49" t="str"/>
       <x:c r="H50" s="49" t="str"/>
       <x:c r="I50" s="49" t="str">
-        <x:f>IF(OR(G50="",H50=""),"",H50-G50)</x:f>
+        <x:f>IF(AND(ISNUMBER(G50),ISNUMBER(H50),G50&gt;=0,H50&gt;=0),H50-G50,"")</x:f>
       </x:c>
       <x:c r="J50" s="53" t="str">
-        <x:f>IF(OR(G50="",H50=""),"",IF(G50=0,IF(H50=0,0,1),I50/G50))</x:f>
+        <x:f>IF(ISNUMBER(I50),IF(G50=0,"N/A",I50/G50),"")</x:f>
       </x:c>
       <x:c r="K50" s="57" t="str"/>
       <x:c r="L50" s="57" t="str">
-        <x:f>IF(OR(I50="",K50=""),"",I50*K50)</x:f>
+        <x:f>IF(AND(ISNUMBER(I50),ISNUMBER(K50),K50&gt;=0),I50*K50,"")</x:f>
       </x:c>
       <x:c r="M50" s="42" t="str">
-        <x:f>IF(I50="","",IF(I50=0,"MATCHED",IF(I50&lt;0,"SHORTAGE","EXCESS")))</x:f>
+        <x:f>IF(COUNTA(B50:H50,K50)=0,"",IF(ISNUMBER(I50),IF(I50=0,"MATCHED",IF(I50&lt;0,"SHORTAGE","EXCESS")),"INCOMPLETE"))</x:f>
       </x:c>
     </x:row>
     <x:row r="51">
@@ -1677,17 +1717,17 @@
       <x:c r="G51" s="48" t="str"/>
       <x:c r="H51" s="48" t="str"/>
       <x:c r="I51" s="48" t="str">
-        <x:f>IF(OR(G51="",H51=""),"",H51-G51)</x:f>
+        <x:f>IF(AND(ISNUMBER(G51),ISNUMBER(H51),G51&gt;=0,H51&gt;=0),H51-G51,"")</x:f>
       </x:c>
       <x:c r="J51" s="52" t="str">
-        <x:f>IF(OR(G51="",H51=""),"",IF(G51=0,IF(H51=0,0,1),I51/G51))</x:f>
+        <x:f>IF(ISNUMBER(I51),IF(G51=0,"N/A",I51/G51),"")</x:f>
       </x:c>
       <x:c r="K51" s="56" t="str"/>
       <x:c r="L51" s="56" t="str">
-        <x:f>IF(OR(I51="",K51=""),"",I51*K51)</x:f>
+        <x:f>IF(AND(ISNUMBER(I51),ISNUMBER(K51),K51&gt;=0),I51*K51,"")</x:f>
       </x:c>
       <x:c r="M51" s="40" t="str">
-        <x:f>IF(I51="","",IF(I51=0,"MATCHED",IF(I51&lt;0,"SHORTAGE","EXCESS")))</x:f>
+        <x:f>IF(COUNTA(B51:H51,K51)=0,"",IF(ISNUMBER(I51),IF(I51=0,"MATCHED",IF(I51&lt;0,"SHORTAGE","EXCESS")),"INCOMPLETE"))</x:f>
       </x:c>
     </x:row>
     <x:row r="52">
@@ -1702,17 +1742,17 @@
       <x:c r="G52" s="49" t="str"/>
       <x:c r="H52" s="49" t="str"/>
       <x:c r="I52" s="49" t="str">
-        <x:f>IF(OR(G52="",H52=""),"",H52-G52)</x:f>
+        <x:f>IF(AND(ISNUMBER(G52),ISNUMBER(H52),G52&gt;=0,H52&gt;=0),H52-G52,"")</x:f>
       </x:c>
       <x:c r="J52" s="53" t="str">
-        <x:f>IF(OR(G52="",H52=""),"",IF(G52=0,IF(H52=0,0,1),I52/G52))</x:f>
+        <x:f>IF(ISNUMBER(I52),IF(G52=0,"N/A",I52/G52),"")</x:f>
       </x:c>
       <x:c r="K52" s="57" t="str"/>
       <x:c r="L52" s="57" t="str">
-        <x:f>IF(OR(I52="",K52=""),"",I52*K52)</x:f>
+        <x:f>IF(AND(ISNUMBER(I52),ISNUMBER(K52),K52&gt;=0),I52*K52,"")</x:f>
       </x:c>
       <x:c r="M52" s="42" t="str">
-        <x:f>IF(I52="","",IF(I52=0,"MATCHED",IF(I52&lt;0,"SHORTAGE","EXCESS")))</x:f>
+        <x:f>IF(COUNTA(B52:H52,K52)=0,"",IF(ISNUMBER(I52),IF(I52=0,"MATCHED",IF(I52&lt;0,"SHORTAGE","EXCESS")),"INCOMPLETE"))</x:f>
       </x:c>
     </x:row>
     <x:row r="55">
@@ -1970,6 +2010,7 @@
     <x:mergeCell ref="A70:D71"/>
     <x:mergeCell ref="E70:H71"/>
     <x:mergeCell ref="I70:M71"/>
+    <x:mergeCell ref="A10:M10"/>
   </x:mergeCells>
   <x:conditionalFormatting sqref="M13:M52">
     <x:cfRule type="expression" dxfId="0" priority="1">
@@ -1981,10 +2022,11 @@
     <x:cfRule type="expression" dxfId="2" priority="3">
       <x:formula>M13="EXCESS"</x:formula>
     </x:cfRule>
+    <x:cfRule type="containsText" dxfId="3" priority="4" operator="containsText" text="INCOMPLETE"/>
   </x:conditionalFormatting>
   <x:dataValidations count="2">
     <x:dataValidation type="list" sqref="B5">
-      <x:formula1>"QAR,USD,EUR,GBP,AED,SAR,LKR,INR"</x:formula1>
+      <x:formula1>"USD,EUR,GBP,CAD,AUD,NZD,CHF,JPY,CNY,HKD,SGD,INR,AED,SAR,QAR,LKR,ZAR,BRL,MXN"</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="F13:F52">
       <x:formula1>"PCS,EA,BOX,CTN,KG,G,L,ML,M,SET,PACK"</x:formula1>
@@ -2002,7 +2044,7 @@
     <x:col min="2" max="2" width="82" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
-    <x:row r="1">
+    <x:row r="1" ht="30" customHeight="1">
       <x:c r="A1" s="65" t="str">
         <x:v>DIXANI Stock Variance Report - How to Use</x:v>
       </x:c>
@@ -2012,81 +2054,126 @@
       <x:c r="E1" s="65"/>
       <x:c r="F1" s="65"/>
     </x:row>
-    <x:row r="3" ht="34" customHeight="1">
-      <x:c r="A3" s="44" t="str">
+    <x:row r="3" ht="56" customHeight="1">
+      <x:c r="A3" s="70" t="str">
         <x:v>Purpose</x:v>
       </x:c>
-      <x:c r="B3" s="40" t="str">
+      <x:c r="B3" s="71" t="str">
         <x:v>Compare system stock with a completed physical count and document inventory discrepancies.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="4" ht="34" customHeight="1">
-      <x:c r="A4" s="44" t="str">
+      <x:c r="C3" s="71"/>
+      <x:c r="D3" s="71"/>
+      <x:c r="E3" s="71"/>
+      <x:c r="F3" s="71"/>
+    </x:row>
+    <x:row r="4" ht="56" customHeight="1">
+      <x:c r="A4" s="70" t="str">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="B4" s="40" t="str">
-        <x:v>Complete the report information at the top of the Variance Report sheet.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="5" ht="34" customHeight="1">
-      <x:c r="A5" s="44" t="str">
+      <x:c r="B4" s="71" t="str">
+        <x:v>Choose the report currency (USD by default). All unit costs must use that currency. The selector does not convert exchange rates.</x:v>
+      </x:c>
+      <x:c r="C4" s="71"/>
+      <x:c r="D4" s="71"/>
+      <x:c r="E4" s="71"/>
+      <x:c r="F4" s="71"/>
+    </x:row>
+    <x:row r="5" ht="56" customHeight="1">
+      <x:c r="A5" s="70" t="str">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="B5" s="40" t="str">
-        <x:v>Enter SKU, description, category, location, UOM, System Qty, Physical Qty and Unit Cost.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="6" ht="34" customHeight="1">
-      <x:c r="A6" s="44" t="str">
+      <x:c r="B5" s="71" t="str">
+        <x:v>Use rows 13–52. Enter SKU, description, category, location, UOM, system quantity, physical quantity and unit cost. Compare the same item, unit and count cut-off.</x:v>
+      </x:c>
+      <x:c r="C5" s="71"/>
+      <x:c r="D5" s="71"/>
+      <x:c r="E5" s="71"/>
+      <x:c r="F5" s="71"/>
+    </x:row>
+    <x:row r="6" ht="56" customHeight="1">
+      <x:c r="A6" s="70" t="str">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="B6" s="40" t="str">
-        <x:v>Variance Qty is calculated automatically as Physical Qty - System Qty.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="7" ht="34" customHeight="1">
-      <x:c r="A7" s="44" t="str">
+      <x:c r="B6" s="71" t="str">
+        <x:v>Variance quantity = physical quantity minus system quantity. Blank or nonnumeric quantities are unknown. Enter zero only when confirmed. Negative inputs are not accepted by calculations.</x:v>
+      </x:c>
+      <x:c r="C6" s="71"/>
+      <x:c r="D6" s="71"/>
+      <x:c r="E6" s="71"/>
+      <x:c r="F6" s="71"/>
+    </x:row>
+    <x:row r="7" ht="56" customHeight="1">
+      <x:c r="A7" s="70" t="str">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="B7" s="40" t="str">
-        <x:v>Variance % is calculated against System Qty. If System Qty is zero and Physical Qty is positive, the workbook shows 100% as a practical flag.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="8" ht="34" customHeight="1">
-      <x:c r="A8" s="44" t="str">
+      <x:c r="B7" s="71" t="str">
+        <x:v>Variance % = variance quantity / system quantity. A zero system quantity shows N/A, including when both quantities are zero. It is not a 100% variance.</x:v>
+      </x:c>
+      <x:c r="C7" s="71"/>
+      <x:c r="D7" s="71"/>
+      <x:c r="E7" s="71"/>
+      <x:c r="F7" s="71"/>
+    </x:row>
+    <x:row r="8" ht="56" customHeight="1">
+      <x:c r="A8" s="70" t="str">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="B8" s="40" t="str">
-        <x:v>Variance Value = Variance Qty x Unit Cost. Negative values are shortages; positive values are excess.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="9" ht="34" customHeight="1">
-      <x:c r="A9" s="44" t="str">
+      <x:c r="B8" s="71" t="str">
+        <x:v>Variance value = variance quantity x unit cost. All value totals show Incomplete until each started row has valid quantities and a nonnegative numeric cost. A confirmed zero cost is allowed.</x:v>
+      </x:c>
+      <x:c r="C8" s="71"/>
+      <x:c r="D8" s="71"/>
+      <x:c r="E8" s="71"/>
+      <x:c r="F8" s="71"/>
+    </x:row>
+    <x:row r="9" ht="56" customHeight="1">
+      <x:c r="A9" s="70" t="str">
         <x:v>6</x:v>
       </x:c>
-      <x:c r="B9" s="40" t="str">
-        <x:v>Status is assigned automatically as MATCHED, SHORTAGE or EXCESS.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="10" ht="34" customHeight="1">
-      <x:c r="A10" s="44" t="str">
+      <x:c r="B9" s="71" t="str">
+        <x:v>Started Rows counts rows with inputs. MATCHED, SHORTAGE and EXCESS classify valid quantity pairs. INCOMPLETE means quantities need attention. A matched quantity does not confirm cost completeness.</x:v>
+      </x:c>
+      <x:c r="C9" s="71"/>
+      <x:c r="D9" s="71"/>
+      <x:c r="E9" s="71"/>
+      <x:c r="F9" s="71"/>
+    </x:row>
+    <x:row r="10" ht="56" customHeight="1">
+      <x:c r="A10" s="70" t="str">
         <x:v>7</x:v>
       </x:c>
-      <x:c r="B10" s="40" t="str">
-        <x:v>Use the investigation section for reason/root cause, corrective action, owner, due date and approval notes.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="11" ht="34" customHeight="1">
-      <x:c r="A11" s="44" t="str">
+      <x:c r="B10" s="71" t="str">
+        <x:v>Record evidence, corrective action, owner, due date and approvals in the investigation section. Net value offsets shortages against excesses; review both separately.</x:v>
+      </x:c>
+      <x:c r="C10" s="71"/>
+      <x:c r="D10" s="71"/>
+      <x:c r="E10" s="71"/>
+      <x:c r="F10" s="71"/>
+    </x:row>
+    <x:row r="11" ht="56" customHeight="1">
+      <x:c r="A11" s="70" t="str">
         <x:v>Control note</x:v>
       </x:c>
-      <x:c r="B11" s="40" t="str">
-        <x:v>Recount material variances and review transactions before making any approved system adjustment.</x:v>
-      </x:c>
+      <x:c r="B11" s="71" t="str">
+        <x:v>Recount and review transactions before adjustment. Keep each SKU, location and UOM comparison on its own row. Do not duplicate a count or mix currencies. Example values are fictional.</x:v>
+      </x:c>
+      <x:c r="C11" s="71"/>
+      <x:c r="D11" s="71"/>
+      <x:c r="E11" s="71"/>
+      <x:c r="F11" s="71"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:F1"/>
+    <x:mergeCell ref="B3:F3"/>
+    <x:mergeCell ref="B4:F4"/>
+    <x:mergeCell ref="B5:F5"/>
+    <x:mergeCell ref="B6:F6"/>
+    <x:mergeCell ref="B7:F7"/>
+    <x:mergeCell ref="B8:F8"/>
+    <x:mergeCell ref="B9:F9"/>
+    <x:mergeCell ref="B10:F10"/>
+    <x:mergeCell ref="B11:F11"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>